<commit_message>
Proyección y estado metas adquirencia 1 a 1 y wompi hasta 202607
</commit_message>
<xml_diff>
--- a/main_data/df_primer_dia_ing_vinc.xlsx
+++ b/main_data/df_primer_dia_ing_vinc.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1206,6 +1206,34 @@
         <v>778965</v>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B56" t="n">
+        <v>7</v>
+      </c>
+      <c r="C56" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" t="n">
+        <v>783909</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B57" t="n">
+        <v>8</v>
+      </c>
+      <c r="C57" t="n">
+        <v>3</v>
+      </c>
+      <c r="D57" t="n">
+        <v>790026</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar historico transacciones y métricas hasta 202608 tanto de wompi como adquirencia
</commit_message>
<xml_diff>
--- a/main_data/df_primer_dia_ing_vinc.xlsx
+++ b/main_data/df_primer_dia_ing_vinc.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D57"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1234,6 +1234,20 @@
         <v>790026</v>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B58" t="n">
+        <v>9</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
+        <v>795866</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>